<commit_message>
Regenerate CO2 T&S scale sweep on 551 basis; correct false-drift claim
- tea_scale_up_co2ts.py: repoint feedstock files from Jones_572_2MC to the 551
  set (the report/manuscript basis).
- _Scale_Up_Sensitivity.md section 6: 551-basis MJSP table; no-T&S CCS-60% now
  reproduces sections 3c/4 (1.845/0.931/0.803 at 1x/10x/30x). T&S adder unchanged
  (~0.0046 $/L per $1/tCO2, flat across scale).
- section 7 + log: the earlier '3c/4 drift' was a wrong-file comparison (Jones vs
  551), not code drift; corrected. Only pre-fix sections 1/2/3b remain outdated by
  the six-tenths fix.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MjFwwDgUpjrZDZMd1ma7x
</commit_message>
<xml_diff>
--- a/Figure/scale_up_co2ts.xlsx
+++ b/Figure/scale_up_co2ts.xlsx
@@ -475,25 +475,25 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>1.94234683378116</v>
+        <v>1.845068955589855</v>
       </c>
       <c r="C2" t="n">
-        <v>1.960692901286165</v>
+        <v>1.863332753088182</v>
       </c>
       <c r="D2" t="n">
-        <v>2.148740093212463</v>
+        <v>2.050536677446028</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01834606750500445</v>
+        <v>0.01826379749832685</v>
       </c>
       <c r="F2" t="n">
-        <v>0.2063932594313025</v>
+        <v>0.2054677218561729</v>
       </c>
       <c r="G2" t="n">
-        <v>260459.7422965531</v>
+        <v>259508.8407793048</v>
       </c>
       <c r="H2" t="n">
-        <v>56788135.59919688</v>
+        <v>56835680.70727426</v>
       </c>
     </row>
     <row r="3">
@@ -501,25 +501,25 @@
         <v>2.5</v>
       </c>
       <c r="B3" t="n">
-        <v>1.478544284431743</v>
+        <v>1.436693830318925</v>
       </c>
       <c r="C3" t="n">
-        <v>1.496888453768995</v>
+        <v>1.454957627543894</v>
       </c>
       <c r="D3" t="n">
-        <v>1.684916189475828</v>
+        <v>1.642161549099817</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01834416933725258</v>
+        <v>0.0182637972249684</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2063719050440855</v>
+        <v>0.205467718780892</v>
       </c>
       <c r="G3" t="n">
-        <v>651180.6365367799</v>
+        <v>648772.0973948891</v>
       </c>
       <c r="H3" t="n">
-        <v>141991850.285505</v>
+        <v>142089202.8976218</v>
       </c>
     </row>
     <row r="4">
@@ -527,25 +527,25 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1.317093196286278</v>
+        <v>1.178218941449239</v>
       </c>
       <c r="C4" t="n">
-        <v>1.335404207902641</v>
+        <v>1.196482738674207</v>
       </c>
       <c r="D4" t="n">
-        <v>1.52309207697036</v>
+        <v>1.383686660230132</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0183110116163625</v>
+        <v>0.01826379722496818</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2059988806840816</v>
+        <v>0.2054677187808931</v>
       </c>
       <c r="G4" t="n">
-        <v>1303587.29459718</v>
+        <v>1297544.194789761</v>
       </c>
       <c r="H4" t="n">
-        <v>284765762.1345857</v>
+        <v>284178405.7952431</v>
       </c>
     </row>
     <row r="5">
@@ -553,25 +553,25 @@
         <v>7.5</v>
       </c>
       <c r="B5" t="n">
-        <v>1.248122208645362</v>
+        <v>1.040315250120718</v>
       </c>
       <c r="C5" t="n">
-        <v>1.26646056141932</v>
+        <v>1.058579042876484</v>
       </c>
       <c r="D5" t="n">
-        <v>1.454428677352388</v>
+        <v>1.24578291862308</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01833835277395823</v>
+        <v>0.01826379275576584</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2063064687070266</v>
+        <v>0.2054676685023615</v>
       </c>
       <c r="G5" t="n">
-        <v>1953872.361912718</v>
+        <v>1946316.309556016</v>
       </c>
       <c r="H5" t="n">
-        <v>426182740.8375208</v>
+        <v>426267716.8063174</v>
       </c>
     </row>
     <row r="6">
@@ -579,25 +579,25 @@
         <v>10</v>
       </c>
       <c r="B6" t="n">
-        <v>1.167705278083964</v>
+        <v>0.9314377202680284</v>
       </c>
       <c r="C6" t="n">
-        <v>1.186044015963503</v>
+        <v>0.9497015174238471</v>
       </c>
       <c r="D6" t="n">
-        <v>1.37401607922878</v>
+        <v>1.13690543827099</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01833873787953921</v>
+        <v>0.01826379715581872</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2063108011448156</v>
+        <v>0.2054677180029618</v>
       </c>
       <c r="G6" t="n">
-        <v>2605134.863583922</v>
+        <v>2595088.389580065</v>
       </c>
       <c r="H6" t="n">
-        <v>568225551.9864336</v>
+        <v>568356813.7424891</v>
       </c>
     </row>
     <row r="7">
@@ -605,25 +605,25 @@
         <v>20</v>
       </c>
       <c r="B7" t="n">
-        <v>1.031962686023721</v>
+        <v>0.8437690196521511</v>
       </c>
       <c r="C7" t="n">
-        <v>1.050302391603007</v>
+        <v>0.8620328124081124</v>
       </c>
       <c r="D7" t="n">
-        <v>1.238284373790678</v>
+        <v>1.049236688156714</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01833970557928533</v>
+        <v>0.01826379275596124</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2063216877669567</v>
+        <v>0.2054676685045626</v>
       </c>
       <c r="G7" t="n">
-        <v>5210125.78230099</v>
+        <v>5190176.82545804</v>
       </c>
       <c r="H7" t="n">
-        <v>1136359743.5688</v>
+        <v>1136713911.465949</v>
       </c>
     </row>
     <row r="8">
@@ -631,25 +631,25 @@
         <v>30</v>
       </c>
       <c r="B8" t="n">
-        <v>0.9357864622194375</v>
+        <v>0.8024808016204954</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9541266285752052</v>
+        <v>0.8207445987765002</v>
       </c>
       <c r="D8" t="n">
-        <v>1.142113333721822</v>
+        <v>1.007948519625547</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01834016635576774</v>
+        <v>0.01826379715600479</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2063268715023844</v>
+        <v>0.2054677180050519</v>
       </c>
       <c r="G8" t="n">
-        <v>7815087.605188597</v>
+        <v>7785265.16869856</v>
       </c>
       <c r="H8" t="n">
-        <v>1704474747.630815</v>
+        <v>1705070441.200977</v>
       </c>
     </row>
   </sheetData>

</xml_diff>